<commit_message>
docs: 变更追踪表登记 Batch 4 租约统一与 CI PG（C-199/C-200/C-201）
重跑 generate_change_log.py（201 rows）与 build_prd_html.py（28 PRDs）
对齐改动表与 PRD.html
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N200"/>
+  <dimension ref="A1:N203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14845,8 +14845,224 @@
         </is>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08 11:01</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>C-199</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>bb8af94</t>
+        </is>
+      </c>
+      <c r="E201" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F201" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G201" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H201" s="5" t="inlineStr">
+        <is>
+          <t>docs: 变更追踪表登记 Batch 3 分布式限流 fix（C-197/C-198）</t>
+        </is>
+      </c>
+      <c r="I201" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J201" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K201" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L201" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M201" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N201" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08 17:23</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>C-200</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D202" s="4" t="inlineStr">
+        <is>
+          <t>7d31056</t>
+        </is>
+      </c>
+      <c r="E202" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F202" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G202" s="5" t="inlineStr">
+        <is>
+          <t>后端</t>
+        </is>
+      </c>
+      <c r="H202" s="5" t="inlineStr">
+        <is>
+          <t>refactor: 统一任务级执行租约到 task_lease.py，收敛 execution_token 写点并补协作取消（A4）</t>
+        </is>
+      </c>
+      <c r="I202" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J202" s="5" t="inlineStr">
+        <is>
+          <t>backend/app/core；backend/app/services；backend/app/worker.py；backend/tests/test_dag_workflow.py；backend/tests/test_orchestrator.py；backend/tests/test_worker_lease.py</t>
+        </is>
+      </c>
+      <c r="K202" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L202" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M202" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N202" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08 17:23</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>C-201</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>bc2adeb</t>
+        </is>
+      </c>
+      <c r="E203" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F203" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G203" s="5" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="H203" s="5" t="inlineStr">
+        <is>
+          <t>optimize: CI 增加 PostgreSQL + Redis job 与前端 lint/test job（A3）</t>
+        </is>
+      </c>
+      <c r="I203" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J203" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K203" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L203" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M203" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N203" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N200"/>
+  <autoFilter ref="A2:N203"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -15049,6 +15265,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId196"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId197"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId201"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: 登记 Batch 7/8 回写与 OPT-3/OPT-4 并重生成（C-206~C-210）
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$212</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N208"/>
+  <dimension ref="A1:N212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15421,8 +15421,296 @@
         </is>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:38</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>C-207</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D209" s="4" t="inlineStr">
+        <is>
+          <t>41b3470</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F209" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G209" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H209" s="5" t="inlineStr">
+        <is>
+          <t>docs: 回填 C-193~C-201 改动内容与验收结论并重生成变更追踪表</t>
+        </is>
+      </c>
+      <c r="I209" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J209" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K209" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L209" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M209" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N209" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:44</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>C-208</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>3b1aa8b</t>
+        </is>
+      </c>
+      <c r="E210" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F210" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G210" s="5" t="inlineStr">
+        <is>
+          <t>部署</t>
+        </is>
+      </c>
+      <c r="H210" s="5" t="inlineStr">
+        <is>
+          <t>docker-compose 三处硬编码 user: "0:0" 改为 ${COMPOSE_USER:-0:0}，生产可用环境变量覆盖 root 运行（20260907 报告 D5 / OPT-4）</t>
+        </is>
+      </c>
+      <c r="I210" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J210" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K210" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L210" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M210" s="5" t="inlineStr">
+        <is>
+          <t>docker compose config 解析通过，未设变量时仍得 user '0:0'（向后兼容）</t>
+        </is>
+      </c>
+      <c r="N210" s="5" t="inlineStr">
+        <is>
+          <t>覆盖 api/worker/frontend 三服务；默认行为不变</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:44</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>C-209</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>a49fa6d</t>
+        </is>
+      </c>
+      <c r="E211" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F211" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G211" s="5" t="inlineStr">
+        <is>
+          <t>文档、其他</t>
+        </is>
+      </c>
+      <c r="H211" s="5" t="inlineStr">
+        <is>
+          <t>Batch 7 文档回写：修正 README 测试数（230/40→245/41）、HANDOFF 更新时间/剩余缺口/架构图服务清单/测试基准、项目计划 Phase 3 状态与表数（20→21）及核查日期、PRD.md 链接多余 docs/ 前缀；并回写 0828/0907 两份审查报告的已完成项状态</t>
+        </is>
+      </c>
+      <c r="I211" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J211" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K211" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L211" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M211" s="5" t="inlineStr">
+        <is>
+          <t>重跑生成脚本无额外差异；PRD.html 由 PRD.md 重生成，索引链接可达</t>
+        </is>
+      </c>
+      <c r="N211" s="5" t="inlineStr">
+        <is>
+          <t>纯文档；覆盖 20260924 审核报告 §四 的 13 处偏差（其中 PRODUCT.md 语言项经核实为误报，未改）</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:44</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>C-210</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D212" s="4" t="inlineStr">
+        <is>
+          <t>ed43106</t>
+        </is>
+      </c>
+      <c r="E212" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F212" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G212" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="H212" s="5" t="inlineStr">
+        <is>
+          <t>applySnapshotTasks 追加快照中 current 缺失的新任务：此前仅按 id 合并已有任务、丢弃快照新增任务，重连对账时其他客户端新建的任务不下发（20260907 报告 C5 / OPT-3）</t>
+        </is>
+      </c>
+      <c r="I212" s="5" t="inlineStr">
+        <is>
+          <t>lib/task-utils.ts applySnapshotTasks 新增 appended（按 id 去重过滤快照新任务后 concat）；tests/task-utils.test.mjs 反向用例改为「追加快照新任务」并补空快照引用不变用例</t>
+        </is>
+      </c>
+      <c r="J212" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K212" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L212" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M212" s="5" t="inlineStr">
+        <is>
+          <t>前端 npm test 35 passed/0 failed（原 34，净增 1）；npm run lint 0 错误；npm run build 成功</t>
+        </is>
+      </c>
+      <c r="N212" s="5" t="inlineStr">
+        <is>
+          <t>消费方 hooks/use-tasks.ts:152 断线快照对账；返回引用不变的语义仅在快照为空时保持</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N208"/>
+  <autoFilter ref="A2:N212"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -15633,6 +15921,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId204"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId205"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId210"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>